<commit_message>
New Firmware and script
Firmware revamp with Support for XBMC4Gamers
</commit_message>
<xml_diff>
--- a/PCB/PicknPlace.xlsx
+++ b/PCB/PicknPlace.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="PickAndPlace_OXFP_2025-08-18" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="PickAndPlace_OXFP_2025-08-22" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="74">
   <si>
     <t>Designator</t>
   </si>
@@ -181,7 +181,16 @@
     <t>POWER</t>
   </si>
   <si>
-    <t>-34.568mm</t>
+    <t>37.719mm</t>
+  </si>
+  <si>
+    <t>-36.449mm</t>
+  </si>
+  <si>
+    <t>34.469mm</t>
+  </si>
+  <si>
+    <t>-34.949mm</t>
   </si>
   <si>
     <t>GND</t>
@@ -925,22 +934,22 @@
         <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="H8" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -960,7 +969,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
@@ -969,22 +978,22 @@
         <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -1004,31 +1013,31 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J10">
         <v>5</v>
@@ -1043,36 +1052,36 @@
         <v>20</v>
       </c>
       <c r="N10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J11">
         <v>5</v>
@@ -1087,7 +1096,7 @@
         <v>20</v>
       </c>
       <c r="N11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>